<commit_message>
scan: seg7 2026-10-09 00:28 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>68.30025567501946</v>
+        <v>68.30025571171281</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>33.19802487298343</v>
+        <v>33.19802482374598</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.26964248233401</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.546822453499203</v>
+        <v>2.546822453387924</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>73.00506740324394</v>
+        <v>73.00506742630668</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>24.71143669598037</v>
+        <v>24.7114367203924</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.645293456559082</v>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>63.64468419942062</v>
+        <v>63.64468416348584</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>30.53825023539732</v>
+        <v>30.53825025174885</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.5057604137868421</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4.588242928023369</v>
+        <v>4.588242932140446</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>820.8298885970225</v>
+        <v>820.8298885970227</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>173.5</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>64.78453536660777</v>
+        <v>64.78453538533606</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>31.3513241532587</v>
+        <v>31.35132417096243</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.023442914175309</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.370630322081094</v>
+        <v>1.370630324417784</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>813.0447459411859</v>
+        <v>813.0447459411863</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>75.5</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>56.03333000774683</v>
+        <v>56.03333013034994</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>30.85126065835068</v>
+        <v>30.85126068890854</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.095572866015456</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-0.0175237084919384</v>
+        <v>-0.0175237087367255</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>809.7372899833889</v>
+        <v>809.7372899833891</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>290</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65.04093581225301</v>
+        <v>65.04093578466254</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>35.12573308579461</v>
+        <v>35.12573303754017</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.422533389623288</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3.137175744656668</v>
+        <v>3.137175744211621</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>790.1222362393586</v>
+        <v>790.1222362393592</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>169</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>67.39225428042852</v>
+        <v>67.3922541577777</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>16.25538784782221</v>
+        <v>16.25538788714486</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.66458457284631</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.8624186492978421</v>
+        <v>0.862418649275591</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>778.0107053407772</v>
+        <v>778.0107053407771</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1620</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>56.62039667324853</v>
+        <v>56.62039668583535</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14.58119228194667</v>
+        <v>14.58119230886186</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.065498952271493</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>12.73734314445588</v>
+        <v>12.73734314946303</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>48.03806536611751</v>
+        <v>48.03806537892974</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>11.66839844781463</v>
+        <v>11.66839853344686</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.6251586372753443</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>6.806323723606482</v>
+        <v>6.806323720268182</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>62.37177602408506</v>
+        <v>62.3717760838918</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>26.67515218570254</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.2454587996442434</v>
+        <v>0.2454587995886089</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.10022646750414</v>
+        <v>58.10022652079883</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>15.91037556424683</v>
+        <v>15.91037579411765</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.405613130987792</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.0115305362175695</v>
+        <v>-0.0115305366181509</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>65.47784112738451</v>
+        <v>65.47784109092586</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>37.89167415240225</v>
+        <v>37.89167415626235</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.692540222135665</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.682818299311292</v>
+        <v>1.682818299533832</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>51.3536361519407</v>
+        <v>51.35363612400082</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>21.81221480506677</v>
+        <v>21.81221478555909</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.538891473202957</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.07403585766807</v>
+        <v>2.07403585844694</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>707.3233206177961</v>
+        <v>707.323320617796</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>860</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>67.71380029357334</v>
+        <v>67.71380031321391</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>31.79586757951916</v>
+        <v>31.79586756023159</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.987411952912247</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>18.3143392433503</v>
+        <v>18.31433924368408</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>61.02226213758544</v>
+        <v>61.02226216612683</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>54.51874167787732</v>
+        <v>54.51874169135445</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.9145135998959624</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.0967420642693923</v>
+        <v>0.09674206360178771</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.35977203112003</v>
+        <v>54.35977203733256</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>38.16402763854106</v>
+        <v>38.16402767602225</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.3200459778781448</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.2402635987312606</v>
+        <v>-0.2402635989315698</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>651.9504805942468</v>
+        <v>651.9504805942469</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>43.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>56.70677315593453</v>
+        <v>56.70677309923732</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>24.59688790608451</v>
+        <v>24.59688785513037</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5897279548633712</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.1923825266769956</v>
+        <v>0.1923825267660134</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.09817182013013</v>
+        <v>56.098171747103</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.87813926077992</v>
+        <v>32.87813929412277</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.3955200080503376</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-2.037741821764952</v>
+        <v>-2.037741820652236</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>640.2952283599381</v>
+        <v>640.2952283599373</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>146.5</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59.0827618547199</v>
+        <v>59.08276166779534</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>18.30186786608897</v>
+        <v>18.30186785524662</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.089615998888966</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.436428556074849</v>
+        <v>1.436428555741018</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>55.25601582224299</v>
+        <v>55.25602336107279</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>19.06784809717696</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.0433159565243497</v>
+        <v>0.0433159544054649</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>55.97026059283979</v>
+        <v>55.97026068661553</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>31.70808506740269</v>
+        <v>31.70808516180761</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.6883041543283634</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.3611601260583148</v>
+        <v>-0.3611601227201575</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>625.2014958686217</v>
+        <v>625.2014958686218</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>326.5</v>
@@ -1721,7 +1721,7 @@
         <v>59.49119232168679</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>17.63737861149632</v>
+        <v>17.63737859206307</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.7281093378296306</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3.314369692912975</v>
+        <v>3.314369693691855</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>63.67598399092552</v>
+        <v>63.6759839511564</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>45.72243642250884</v>
+        <v>45.72243651116761</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.3587674869748</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-1.57240320649953</v>
+        <v>-1.572403205498119</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>62.48682362270345</v>
+        <v>62.48682379828081</v>
       </c>
       <c r="I26" s="2" t="n">
         <v>23.67342784727498</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.688443483392294</v>
+        <v>1.688443483503576</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>54.96607153724936</v>
+        <v>54.96607149747078</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>29.22796353605459</v>
+        <v>29.22796355665482</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.7903083745296995</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.8654904444320701</v>
+        <v>-0.8654904442317868</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>60.90052520677438</v>
+        <v>60.90052519303752</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>44.88368264772692</v>
+        <v>44.88368271130497</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.230395009067462</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-1.40640780398121</v>
+        <v>-1.406407804648879</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63.01839513091681</v>
+        <v>63.01839508535334</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.14091874516246</v>
+        <v>28.1409187782902</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.3927469016852034</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.344996295171073</v>
+        <v>3.344996295282354</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>51.99035271178772</v>
+        <v>51.99035273060908</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>21.1279084682024</v>
+        <v>21.12790843350702</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.5617434665933119</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>4.607443414263759</v>
+        <v>4.607443415932835</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>50.32166299696349</v>
+        <v>50.32166311856905</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.3317914823519</v>
+        <v>26.33179156239889</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.774222687508543</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.7718726129569262</v>
+        <v>0.7718726145147148</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.85095253074492</v>
+        <v>44.85095267349352</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>28.52398811413727</v>
+        <v>28.52398819503105</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.766750594038366</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>4.875868212784496</v>
+        <v>4.87586821256194</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>62.04589304489731</v>
+        <v>62.04589302009154</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>30.90514252788164</v>
+        <v>30.90514253123838</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8158209642158555</v>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>565.5829173376903</v>
+        <v>565.5829173376866</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>134</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>56.44081136239846</v>
+        <v>56.44081134705787</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>22.7460529679241</v>
+        <v>22.74605296093773</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.532308627232526</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.330726083132334</v>
+        <v>1.33072608308782</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>564.8162972029896</v>
+        <v>564.8162972029897</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>70.59999999999999</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>57.3469399256148</v>
+        <v>57.34694006221467</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>21.6891132448347</v>
+        <v>21.68911323467621</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6685418709482445</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.2106566995886869</v>
+        <v>0.2106566994774233</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46.82022832145206</v>
+        <v>46.82022827612283</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22.15325656831157</v>
+        <v>22.15325653618891</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.4582312388733967</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.1966203235371948</v>
+        <v>0.1966203243160656</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         <v>49.13325702105323</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>27.69639262360299</v>
+        <v>27.69639249812163</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>3.281118673063335</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0750777364872269</v>
+        <v>0.07507773645384749</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>553.2138948479387</v>
+        <v>553.2138948479388</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>120.5</v>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>56.03150266067643</v>
+        <v>56.03150271051428</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>39.46914842950033</v>
+        <v>39.4691484563046</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.352915512131274</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.3078651044215337</v>
+        <v>-0.3078651045327993</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>545.545525135713</v>
+        <v>545.5455251357123</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>161</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>50.58378738862904</v>
+        <v>50.58378769666079</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>16.04703756572491</v>
+        <v>16.04703769564805</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>2.012696041822255</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.3624713325156232</v>
+        <v>0.362471331736701</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>542.0032784378961</v>
+        <v>542.0032784378958</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>291</v>
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>53.55834737859001</v>
+        <v>53.55834735220574</v>
       </c>
       <c r="I40" s="2" t="n">
         <v>11.73143553154014</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1.712435707473815</v>
+        <v>1.712435707251314</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.88650654839083</v>
+        <v>66.88650643458647</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>40.57073608077378</v>
+        <v>40.57073604801951</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.8159300335253036</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>56.42457732823469</v>
+        <v>56.42457758700094</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>28.01751165573507</v>
+        <v>28.01751176996791</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.31935217770055</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.3394497503737149</v>
+        <v>0.3394497498618747</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>535.1167568997715</v>
+        <v>535.1167568997716</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>29.6</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>56.9925908520129</v>
+        <v>56.9925909281676</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>52.78535974790968</v>
+        <v>52.78535992421825</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5155127080805854</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.3354612751422758</v>
+        <v>-0.3354612753425638</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>46.91923705681864</v>
+        <v>46.91923730316898</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>24.70844046508264</v>
+        <v>24.70844046401347</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.271461374968387</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-2.679155120354475</v>
+        <v>-2.679155127475802</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>52.31322566712442</v>
+        <v>52.31322524445017</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.01138582350238</v>
+        <v>27.01138581973479</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.9235230489516928</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.1856464102938567</v>
+        <v>0.1856464109392357</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>44.9991557554707</v>
+        <v>44.9991557421269</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>48.31963542063882</v>
+        <v>48.31963529638239</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.626667126013117</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-5.11957079415383</v>
+        <v>-5.119570793864533</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>527.6531069882661</v>
+        <v>527.6531069882667</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>16.55</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>57.75552099254783</v>
+        <v>57.75552105399233</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>29.9571594400714</v>
+        <v>29.95715948300909</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>2.026691960685566</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.1173573979640883</v>
+        <v>0.1173573979195798</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>44.27047609146121</v>
+        <v>44.27047616232272</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.1559741029023</v>
+        <v>22.15597414396172</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>2.568828275715989</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.6298719085378011</v>
+        <v>-0.6298719089829294</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>49.06363090833889</v>
+        <v>49.06363097964999</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>21.90079752953228</v>
+        <v>21.90079752374312</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4508113287235993</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.2900923615645796</v>
+        <v>-0.2900923612307342</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>45.34092515141356</v>
+        <v>45.34092517800796</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>28.1863956887621</v>
+        <v>28.18639569244968</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5531914363784936</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-2.006864914546561</v>
+        <v>-2.006864914991632</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>515.1638323956149</v>
+        <v>515.163832395615</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>136.5</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.24329563873633</v>
+        <v>45.24329564150688</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>26.83480228283468</v>
+        <v>26.83480229922932</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.5144950983648667</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-2.413068608823476</v>
+        <v>-2.413068608801217</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>513.3878772355463</v>
+        <v>513.3878772355462</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>66.7</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.29662783470428</v>
+        <v>52.29662782544845</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.430786063139971</v>
+        <v>8.430786047328649</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>1.337221909016002</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1.22968448938938</v>
+        <v>1.229684489723195</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>56.72216886930816</v>
+        <v>56.72216893621275</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>33.4035212832373</v>
+        <v>33.40352128468344</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5599382696461727</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>45.10405202585708</v>
+        <v>45.10405205242138</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.22443949168438</v>
+        <v>16.22443952309385</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4564191399267124</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>13.93816890798377</v>
+        <v>13.93816890486824</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>476.3940878282344</v>
+        <v>476.3940878282345</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>152</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>47.35160958564399</v>
+        <v>47.35160953445973</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.10430200127302</v>
+        <v>11.10430200231222</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.7802337605706574</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.400772742038189</v>
+        <v>1.400772741815649</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>60.78868724498047</v>
+        <v>60.78868716198352</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.20011100515467</v>
+        <v>16.20011139271191</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.3037742932108493</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.5184204928469907</v>
+        <v>0.5184204952949485</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>58.34177923427298</v>
+        <v>58.34177907658229</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.45368101698115</v>
+        <v>16.45368095559672</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.450181888168149</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.1163880756560755</v>
+        <v>0.1163880758452372</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>469.4561265196582</v>
+        <v>469.4561265196581</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>65.8</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>43.61479207023935</v>
+        <v>43.61479203807679</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>49.92852363222395</v>
+        <v>49.92852346018392</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.481116714517904</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1741045995198091</v>
+        <v>-0.1741045996310841</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>54.64787311039142</v>
+        <v>54.64787304063724</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>33.17188136366844</v>
+        <v>33.17188141048766</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.1947280560024797</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.6645011371973704</v>
+        <v>-0.6645011376424814</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>54.35215978115209</v>
+        <v>54.35215976944079</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>28.8407370695504</v>
+        <v>28.84073711932333</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.158514133372914</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.963963227153708</v>
+        <v>-0.9639632257071638</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>49.43217808007619</v>
+        <v>49.43217809854505</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>27.98759361646222</v>
+        <v>27.98759371865979</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.6452168589979339</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-1.588588773642027</v>
+        <v>-1.588588773998094</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>47.37334244812129</v>
+        <v>47.37334245576975</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.52282571617446</v>
+        <v>13.52282572285628</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.5882342702749326</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>25.20556947894101</v>
+        <v>25.20556947782829</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>51.24110898904898</v>
+        <v>51.2411090555792</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.93467957313323</v>
+        <v>22.9346796623055</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3903580845066928</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.2972371449964828</v>
+        <v>-0.2972371461091874</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>51.65400781344772</v>
+        <v>51.65400781449942</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>7.633166010055511</v>
+        <v>7.63316600810276</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>2.448835737686534</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-1.240315548412255</v>
+        <v>-1.240315548523521</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,7 +3891,7 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>37.41460655416459</v>
+        <v>37.41460649908875</v>
       </c>
       <c r="I65" s="2" t="n">
         <v>18.51483560138672</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0033127696301406</v>
+        <v>0.0033127696523955</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>52.3195163772785</v>
+        <v>52.31951637530451</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>8.064490700477059</v>
+        <v>8.064490679535579</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>2.733612273361228</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>5.70841967675813</v>
+        <v>5.708419677203208</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>55.44962302667047</v>
+        <v>55.44962309923185</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>26.721431148776</v>
+        <v>26.72143123462655</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5863235811745992</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.53424371177605</v>
+        <v>1.534243710774611</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>45.21522145421169</v>
+        <v>45.21522146617281</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>10.04215187954296</v>
+        <v>10.04215187339321</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.9664782276683432</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-12.17614973678272</v>
+        <v>-12.17614973682719</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>44.63241887966041</v>
+        <v>44.63241900006828</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>8.341395366499661</v>
+        <v>8.341395361994861</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6706850036822366</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.6900375507425518</v>
+        <v>0.6900375520778192</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>47.30882391063282</v>
+        <v>47.30882388330181</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>33.78076398238063</v>
+        <v>33.78076401580392</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5071619627032389</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.6562626395520903</v>
+        <v>0.6562626399081606</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>55.14734066803935</v>
+        <v>55.14734069551594</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>19.09916836393439</v>
+        <v>19.09916842795922</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.23910734439072</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>7.329285921564937</v>
+        <v>7.329285919117096</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>53.04926709197014</v>
+        <v>53.04926730859336</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>23.28141756461672</v>
+        <v>23.28141755937872</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.6774487725893804</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0898305870087249</v>
+        <v>0.08983058689745441</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>387.5545965173492</v>
+        <v>387.5545965173487</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>32.4</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>56.89576345477012</v>
+        <v>56.89576343395816</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.29017026648331</v>
+        <v>16.29017033401312</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.182903369480411</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0582077357770474</v>
+        <v>0.0582077357325422</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>25.99341965635527</v>
+        <v>25.99341964798284</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>45.33118297905935</v>
+        <v>45.33118298914442</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3032416808382552</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>30.34719792136113</v>
+        <v>30.34719791964477</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.01532144626696</v>
+        <v>45.01532160705612</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>35.24889396442487</v>
+        <v>35.2488939890216</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.4375706557492224</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.7429178693400349</v>
+        <v>-0.7429178705640387</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>372.8513531235829</v>
+        <v>372.8513531235837</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>35.1</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>20.90043710782972</v>
+        <v>20.90043540557235</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>37.84849112249545</v>
+        <v>37.84849333884772</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6906092545194831</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.2067563962755889</v>
+        <v>-0.2067563951740039</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>38.48264192169888</v>
+        <v>38.48264195078113</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>24.03951372491281</v>
+        <v>24.03951375320212</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.5075217280688077</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.6425783363001987</v>
+        <v>0.6425783365227451</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>54.11986215375716</v>
+        <v>54.11986194121604</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>15.12464363952784</v>
+        <v>15.12464393489284</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.07401027846782129</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.2464518733245795</v>
+        <v>0.246451873547133</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>336.5194211537602</v>
+        <v>336.51942115376</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>68</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>25.06710658109182</v>
+        <v>25.06710655206301</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>30.2116448773719</v>
+        <v>30.21164487737191</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>3.610773626878688</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0265962107384383</v>
+        <v>-0.0265962107606881</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>330.4019181659309</v>
+        <v>330.4019181659302</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>0</v>
@@ -4845,7 +4845,7 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>23.10910077520096</v>
+        <v>23.10910075921979</v>
       </c>
       <c r="I83" s="2" t="n">
         <v>12.03699505527415</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-5.882050764519691</v>
+        <v>-5.882050763963326</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>328.4508874188895</v>
+        <v>328.4508874188894</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>71.90000000000001</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>58.10563979963054</v>
+        <v>58.10563961013701</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.43545088642768</v>
+        <v>17.43545072926095</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.5736383681643722</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.8632352674754141</v>
+        <v>0.8632352686326438</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>327.0619951924677</v>
+        <v>327.0619951924684</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>1840</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.86182569934056</v>
+        <v>47.86182570795097</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.2683384170106</v>
+        <v>17.26833841371437</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.5460593787290072</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-24.92779222795424</v>
+        <v>-24.92779223118116</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>54.04339064500957</v>
+        <v>54.04339056152293</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.85901550646056</v>
+        <v>12.85901547461113</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.155151093987921</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.016075441958725</v>
+        <v>-0.0160754420700004</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>60.16187499569192</v>
+        <v>60.16187510250462</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>27.02695350597333</v>
+        <v>27.02695347443517</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.4668041039286125</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.5369390308743149</v>
+        <v>0.5369390294277889</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>43.28448761318927</v>
+        <v>43.28448770294646</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.28426112985334</v>
+        <v>10.28426114487976</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.11149836238872</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.3231250057047132</v>
+        <v>0.3231250056379406</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>48.52395925236974</v>
+        <v>48.52396240007624</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>5.580613701046273</v>
+        <v>5.580613666799087</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.4393353859965352</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.8285801706986122</v>
+        <v>0.8285801268576987</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>47.15610154423229</v>
+        <v>47.15610161389711</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.31572275267757</v>
+        <v>19.3157228365921</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.071524287644398</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.08862708942422839</v>
+        <v>0.0886270891126706</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>45.1758985571167</v>
+        <v>45.17589854604216</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.3778668187468</v>
+        <v>15.37786684539092</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.341645067125195</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.6155984228925919</v>
+        <v>0.6155984224475235</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5378,7 +5378,7 @@
         <v>52.22053517459052</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>23.61865602909376</v>
+        <v>23.6186559827066</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.332262405207214</v>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>300.4355119695249</v>
+        <v>300.4355119695252</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>32</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.22292847332996</v>
+        <v>49.222928405739</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.71252836803819</v>
+        <v>17.71252835174026</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.227778012697675</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1468961363763035</v>
+        <v>0.1468961361648818</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>51.05934329381301</v>
+        <v>51.05934307415978</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>26.12438049364331</v>
+        <v>26.12438050794653</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.4846124356905155</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>46.18124482059641</v>
+        <v>46.18124490769684</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>15.15317015963956</v>
+        <v>15.15317010055109</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7489362044903951</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>1.331329734394968</v>
+        <v>1.331329733949858</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>33.14581076064914</v>
+        <v>33.14581101112843</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>29.1196874110111</v>
+        <v>29.11968747946038</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.6038611477836315</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.4468606490437423</v>
+        <v>0.4468606511579089</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,7 +5693,7 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>27.66320162668463</v>
+        <v>27.66320177685313</v>
       </c>
       <c r="I99" s="2" t="n">
         <v>37.63453746505432</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.6567083667771318</v>
+        <v>0.6567083668883904</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>271.0263759076127</v>
+        <v>271.0263759076125</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>25.5</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>49.63981525312118</v>
+        <v>49.6398151206168</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>31.34532794558877</v>
+        <v>31.34532795496529</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.2581483652302438</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.056129182511651</v>
+        <v>-0.0561291824671429</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>30.35305290771115</v>
+        <v>30.35305298364742</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>12.14012066867233</v>
+        <v>12.14012057361857</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.071720830435555</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0958726521939217</v>
+        <v>-0.0958726522606874</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>50.33739510943994</v>
+        <v>50.33739465573956</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>13.73933925802711</v>
+        <v>13.73933934087768</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5751039035078224</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.2913641883711177</v>
+        <v>0.2913641915979833</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>245.2666357244806</v>
+        <v>245.2666357244805</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>36.1</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.24283676620565</v>
+        <v>52.24283705479002</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>14.49921385894385</v>
+        <v>14.49921384830902</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5548265515267909</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.1195131434722324</v>
+        <v>0.1195131433275752</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>41.53131310262876</v>
+        <v>41.53131316305589</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>16.11313988891058</v>
+        <v>16.1131398992769</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.3552683803288763</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.2115559009036962</v>
+        <v>0.2115559010594885</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>236.9843172392924</v>
+        <v>236.9843172392925</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>35.7</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.72470480481031</v>
+        <v>42.72470348661386</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>10.72970306598392</v>
+        <v>10.72970375519665</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.5972683625262174</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.09037625306104489</v>
+        <v>0.0903762533948541</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.18868673035523</v>
+        <v>50.18868659681389</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.67989817959953</v>
+        <v>13.67989814541059</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.2002847541067448</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.3120129113544023</v>
+        <v>-0.312012911376657</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>226.7949030897593</v>
+        <v>226.7949030897586</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>36.85</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>44.3990051847987</v>
+        <v>44.39900535685848</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>35.82132105199927</v>
+        <v>35.821321189104</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.2747177275349578</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.2252338105672952</v>
+        <v>-0.2252338110123831</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>52.11015844914125</v>
+        <v>52.11015844719259</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>8.893518659982117</v>
+        <v>8.893518663665803</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.7715106812434813</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.5391075233381513</v>
+        <v>0.5391075233715303</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.97751023293412</v>
+        <v>40.97751018254605</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>12.25905122460993</v>
+        <v>12.25905121525441</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.4265577258606749</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>43.27636853255283</v>
+        <v>43.27636943110653</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>10.97017253196276</v>
+        <v>10.97017256952574</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.6944112305375483</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0403910980080954</v>
+        <v>0.0403910976742875</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>205.4876869730768</v>
+        <v>205.4876869730767</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>73.59999999999999</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.84103283737736</v>
+        <v>46.84102864760256</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.57422817828689</v>
+        <v>14.5742295487741</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.1950710223370058</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1719860589459398</v>
+        <v>-0.171986044302638</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>200.0762819365941</v>
+        <v>200.0762819365945</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>33.55</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>51.52213766073734</v>
+        <v>51.5221376619051</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>7.360269177357964</v>
+        <v>7.360269190876881</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.6579849211788896</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.7715142106720666</v>
+        <v>0.7715142106831939</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>32.09203593306189</v>
+        <v>32.09203646378026</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>23.00490015882126</v>
+        <v>23.00490010909286</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.2552688175517914</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0811845418081512</v>
+        <v>-0.08118454225323619</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.00215815782613</v>
+        <v>40.00215813912604</v>
       </c>
       <c r="I115" s="2" t="n">
         <v>23.45723825138411</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0666603632790637</v>
+        <v>-0.0666603632901908</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>193.3306779205678</v>
+        <v>193.3306779205685</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>19.45</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>42.96053923140346</v>
+        <v>42.96053927336681</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.17516196475034</v>
+        <v>16.17516194096955</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.4213970566760561</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1293790874077807</v>
+        <v>-0.1293790874522903</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>32.61790752691688</v>
+        <v>32.61790788655175</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>22.48847349482763</v>
+        <v>22.48847364367884</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4749274537933962</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.905784294410012</v>
+        <v>-0.905784294454528</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>183.1426765614593</v>
+        <v>183.1426765614592</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>26.55</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>33.81625975738694</v>
+        <v>33.81625972607885</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.88077071031263</v>
+        <v>23.88077071031264</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.8699004936014489</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0051779719742817</v>
+        <v>0.0051779720076648</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>182.0902416818437</v>
+        <v>182.0902416818425</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>73.40000000000001</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>35.14603263037355</v>
+        <v>35.14603279959668</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>12.99919524639696</v>
+        <v>12.9991952328545</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.8592391715171215</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.2776834150040141</v>
+        <v>-0.2776834154936073</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>152.0196136673981</v>
+        <v>152.0196136673983</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>29.7</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>40.6932935069036</v>
+        <v>40.69329362252756</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>9.546971973779684</v>
+        <v>9.546972003825491</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.9326239046767693</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.008277346963633799</v>
+        <v>0.008277347030397</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>148.3111265158202</v>
+        <v>148.3111265158197</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>50.2</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>53.79102650329644</v>
+        <v>53.79102656575002</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>23.72951669595404</v>
+        <v>23.7295167014878</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.576402959485849</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.072929203771574</v>
+        <v>0.0729292037159404</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>143.3299578381904</v>
+        <v>143.3299578381896</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>166</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>39.38148171281449</v>
+        <v>39.38148185247181</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>17.34568035078376</v>
+        <v>17.34568048489323</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.8422734130354856</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0972389043670443</v>
+        <v>-0.0972389049233979</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>42.00980838938187</v>
+        <v>42.0098083505257</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>16.61728027843434</v>
+        <v>16.6172804228878</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.4252751215884963</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.96245179959467</v>
+        <v>-0.9624517994744924</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>132.9906000589777</v>
+        <v>132.9906000589774</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>45</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>41.88649652890738</v>
+        <v>41.88649615799974</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.57723378760537</v>
+        <v>12.57723380374128</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.4820937980073715</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.08202992315319001</v>
+        <v>-0.0820299223075267</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>51.34344159873033</v>
+        <v>51.34344159048589</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.85018834807398</v>
+        <v>16.85018835316239</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.4189980584367054</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.871040950628917</v>
+        <v>-1.871040951074016</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>85.74396067139773</v>
+        <v>85.7439606713977</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>66.09999999999999</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>40.08590978557161</v>
+        <v>40.08590973427396</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>16.13356695085351</v>
+        <v>16.13356696693544</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.9289307309261348</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.1116062607454018</v>
+        <v>-0.1116062610792103</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>25.10859852701072</v>
+        <v>25.10859848809146</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>16.84372687654241</v>
+        <v>16.84372687654242</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.7619509147415975</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.22910165119318</v>
+        <v>-0.2291016512376877</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>73.60965960820542</v>
+        <v>73.60965960820545</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>17.4</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>32.18038968692312</v>
+        <v>32.18038970384552</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>17.04639732297666</v>
+        <v>17.04639732297665</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>1.376083320559793</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.0434692336334355</v>
+        <v>-0.0434692336111838</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg7 2026-10-10 00:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>68.30025571171281</v>
+        <v>68.30025559779415</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>33.19802482374598</v>
+        <v>33.19802478739227</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.26964248233401</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.546822453387924</v>
+        <v>2.54682245422913</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>63.64468416348584</v>
+        <v>63.64468415111961</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>30.53825025174885</v>
+        <v>30.538250272398</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>0.5057604137868421</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4.588242932140446</v>
+        <v>4.588242932260609</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>820.8298885970227</v>
+        <v>820.8298885970228</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>173.5</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>64.78453538533606</v>
+        <v>64.78453528449144</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>31.35132417096243</v>
+        <v>31.35132420408966</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.023442914175309</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.370630324417784</v>
+        <v>1.370630327301922</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>813.0447459411863</v>
+        <v>813.0447459411859</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>75.5</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>56.03333013034994</v>
+        <v>56.03333007674316</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>30.85126068890854</v>
+        <v>30.85126064896514</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.095572866015456</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-0.0175237087367255</v>
+        <v>-0.0175237087127055</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>809.7372899833891</v>
+        <v>809.7372899833886</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>290</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65.04093578466254</v>
+        <v>65.04093589244513</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>35.12573303754017</v>
+        <v>35.12573307733471</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.422533389623288</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3.137175744211621</v>
+        <v>3.137175743130006</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>790.1222362393592</v>
+        <v>790.122236239359</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>169</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>67.3922541577777</v>
+        <v>67.39225409856698</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>16.25538788714486</v>
+        <v>16.25538797758231</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.66458457284631</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.862418649275591</v>
+        <v>0.8624186485545571</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>778.0107053407771</v>
+        <v>778.0107053407769</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1620</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>56.62039668583535</v>
+        <v>56.62039663949278</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>14.58119230886186</v>
+        <v>14.5811923842494</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.065498952271493</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>12.73734314946303</v>
+        <v>12.73734315775507</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>48.03806537892974</v>
+        <v>48.03806537281864</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>11.66839853344686</v>
+        <v>11.66839863071668</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.6251586372753443</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>6.806323720268182</v>
+        <v>6.806323725075345</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>62.3717760838918</v>
+        <v>62.37177608959767</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>26.67515218570254</v>
+        <v>26.67515219491109</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.938211250016006</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.2454587995886089</v>
+        <v>0.2454587996246595</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>767.631957299106</v>
+        <v>767.6319572991059</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>62.6</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.10022652079883</v>
+        <v>58.10022659541142</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>15.91037579411765</v>
+        <v>15.91037581829636</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.405613130987792</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.0115305366181509</v>
+        <v>-0.011530536930597</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>65.47784109092586</v>
+        <v>65.47784112508333</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>37.89167415626235</v>
+        <v>37.89167416921146</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.692540222135665</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.682818299533832</v>
+        <v>1.682818299173331</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>51.35363612400082</v>
+        <v>51.35363615199889</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>21.81221478555909</v>
+        <v>21.81221487043973</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.538891473202957</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.07403585844694</v>
+        <v>2.074035857605743</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>707.323320617796</v>
+        <v>707.3233206177943</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>860</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>67.71380031321391</v>
+        <v>67.71380030515624</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>31.79586756023159</v>
+        <v>31.79586753105053</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.987411952912247</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>18.31433924368408</v>
+        <v>18.31433924656832</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>61.02226216612683</v>
+        <v>61.02226212951921</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>54.51874169135445</v>
+        <v>54.51874163271945</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.9145135998959624</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.09674206360178771</v>
+        <v>0.0967420644430063</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.35977203733256</v>
+        <v>54.35977204522255</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>38.16402767602225</v>
+        <v>38.16402772057198</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.3200459778781448</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.2402635989315698</v>
+        <v>-0.2402635988834838</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>651.9504805942469</v>
+        <v>651.9504805942468</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>43.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>56.70677309923732</v>
+        <v>56.70677313719531</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>24.59688785513037</v>
+        <v>24.59688787044177</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5897279548633712</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.1923825267660134</v>
+        <v>0.1923825266939087</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.098171747103</v>
+        <v>56.09817175963541</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.87813929412277</v>
+        <v>32.87813933264115</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.3955200080503376</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-2.037741820652236</v>
+        <v>-2.03774182197413</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>640.2952283599373</v>
+        <v>640.2952283599383</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>146.5</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59.08276166779534</v>
+        <v>59.08276180199758</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>18.30186785524662</v>
+        <v>18.30186804670286</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.089615998888966</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.436428555741018</v>
+        <v>1.436428553577913</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>633.3933626968549</v>
+        <v>633.3933626968548</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>16.55</v>
@@ -1615,7 +1615,7 @@
         <v>55.25602336107279</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>19.06784809717696</v>
+        <v>19.06784589638816</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>2.499836371871321</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.0433159544054649</v>
+        <v>0.043315957456656</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>633.2325412880076</v>
+        <v>633.2325412880078</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>202</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>55.97026068661553</v>
+        <v>55.97026051830012</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>31.70808516180761</v>
+        <v>31.70808518474881</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.6883041543283634</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.3611601227201575</v>
+        <v>-0.3611601180334007</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>625.2014958686218</v>
+        <v>625.2014958686207</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>326.5</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>59.49119232168679</v>
+        <v>59.49119230647462</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>17.63737859206307</v>
+        <v>17.63737839349905</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.7281093378296306</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>3.314369693691855</v>
+        <v>3.314369694533049</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>63.6759839511564</v>
+        <v>63.67598393983669</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>45.72243651116761</v>
+        <v>45.72243651584262</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.3587674869748</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-1.572403205498119</v>
+        <v>-1.572403206699853</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>62.48682379828081</v>
+        <v>62.48682364465061</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.67342784727498</v>
+        <v>23.67342797320735</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.7747877939623102</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.688443483503576</v>
+        <v>1.688443487469266</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>54.96607149747078</v>
+        <v>54.9660715021338</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>29.22796355665482</v>
+        <v>29.22796355070363</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.7903083745296995</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.8654904442317868</v>
+        <v>-0.8654904444961833</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>60.90052519303752</v>
+        <v>60.9005252257905</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>44.88368271130497</v>
+        <v>44.88368278034912</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.230395009067462</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-1.406407804648879</v>
+        <v>-1.406407806090897</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63.01839508535334</v>
+        <v>63.01839513821711</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>28.1409187782902</v>
+        <v>28.14091887176629</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.3927469016852034</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.344996295282354</v>
+        <v>3.344996294441114</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>51.99035273060908</v>
+        <v>51.99035267671385</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>21.12790843350702</v>
+        <v>21.12790834354142</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.5617434665933119</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>4.607443415932835</v>
+        <v>4.607443419057375</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>584.525892906333</v>
+        <v>584.5258929063331</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>118.5</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>50.32166311856905</v>
+        <v>50.32166282327346</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.33179156239889</v>
+        <v>26.33179183345952</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.774222687508543</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.7718726145147148</v>
+        <v>0.771872618119902</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.85095267349352</v>
+        <v>44.85095251976426</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>28.52398819503105</v>
+        <v>28.52398832504081</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.766750594038366</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>4.87586821256194</v>
+        <v>4.875868216167156</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>62.04589302009154</v>
+        <v>62.04589304680545</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>30.90514253123838</v>
+        <v>30.90514253334166</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8158209642158555</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>2.374913670620002</v>
+        <v>2.374913670019126</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>565.5829173376866</v>
+        <v>565.5829173376816</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>134</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>56.44081134705787</v>
+        <v>56.44081137005956</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>22.74605296093773</v>
+        <v>22.74605296262613</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.532308627232526</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.33072608308782</v>
+        <v>1.330726082775377</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>564.8162972029897</v>
+        <v>564.8162972029899</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>70.59999999999999</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>57.34694006221467</v>
+        <v>57.34693988393274</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>21.68911323467621</v>
+        <v>21.68911333761294</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6685418709482445</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.2106566994774233</v>
+        <v>0.210656700078285</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>46.82022827612283</v>
+        <v>46.82022809642567</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22.15325653618891</v>
+        <v>22.15325653556473</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.4582312388733967</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.1966203243160656</v>
+        <v>0.1966203247967729</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,7 +2407,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>49.13325702105323</v>
+        <v>49.13325705548447</v>
       </c>
       <c r="I37" s="2" t="n">
         <v>27.69639249812163</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.07507773645384749</v>
+        <v>0.0750777364177968</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>553.2138948479388</v>
+        <v>553.2138948479385</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>120.5</v>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>56.03150271051428</v>
+        <v>56.03150261506562</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>39.4691484563046</v>
+        <v>39.46914853350746</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.352915512131274</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.3078651045327993</v>
+        <v>-0.3078651042924489</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>545.5455251357123</v>
+        <v>545.5455251357137</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>161</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>50.58378769666079</v>
+        <v>50.58378738471622</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>16.04703769564805</v>
+        <v>16.04703769382787</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>2.012696041822255</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.362471331736701</v>
+        <v>0.3624713329384494</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>53.55834735220574</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>11.73143553154014</v>
+        <v>11.73143565722021</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.6740941960844815</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1.712435707251314</v>
+        <v>1.712435706650465</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>66.88650643458647</v>
+        <v>66.88650683018271</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>40.57073604801951</v>
+        <v>40.57073602406773</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.8159300335253036</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.7030193525883464</v>
+        <v>0.7030193518673098</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>56.42457758700094</v>
+        <v>56.42457737645176</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>28.01751176996791</v>
+        <v>28.01751179473652</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.31935217770055</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.3394497498618747</v>
+        <v>0.3394497499099363</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
         <v>56.9925909281676</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>52.78535992421825</v>
+        <v>52.78535993359301</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5155127080805854</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.3354612753425638</v>
+        <v>-0.3354612753305472</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>46.91923730316898</v>
+        <v>46.91923718536936</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>24.70844046401347</v>
+        <v>24.70844060913973</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.271461374968387</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-2.679155127475802</v>
+        <v>-2.679155122428554</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>44.9991557421269</v>
+        <v>44.999155724241</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>48.31963529638239</v>
+        <v>48.31963529532583</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.626667126013117</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-5.119570793864533</v>
+        <v>-5.119570793984714</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>527.6531069882667</v>
+        <v>527.6531069882665</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>16.55</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>57.75552105399233</v>
+        <v>57.75552116289204</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>29.95715948300909</v>
+        <v>29.9571594633524</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>2.026691960685566</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>44.27047616232272</v>
+        <v>44.27047640903694</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.15597414396172</v>
+        <v>22.1559741332373</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>2.568828275715989</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.6298719089829294</v>
+        <v>-0.6298719070601919</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>49.06363097964999</v>
+        <v>49.06363086516102</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>21.90079752374312</v>
+        <v>21.90079759459304</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4508113287235993</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.2900923612307342</v>
+        <v>-0.2900923594281455</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>45.34092517800796</v>
+        <v>45.34092521117089</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>28.18639569244968</v>
+        <v>28.18639578748063</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5531914363784936</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-2.006864914991632</v>
+        <v>-2.006864914871507</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.24329564150688</v>
+        <v>45.24329565194981</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>26.83480229922932</v>
+        <v>26.83480231083145</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.5144950983648667</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-2.413068608801217</v>
+        <v>-2.413068608729138</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>513.3878772355462</v>
+        <v>513.3878772355463</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>66.7</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.29662782544845</v>
+        <v>52.29662782671114</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.430786047328649</v>
+        <v>8.430786114307505</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>1.337221909016002</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1.229684489723195</v>
+        <v>1.22968448948285</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>56.72216893621275</v>
+        <v>56.72216882874896</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>33.40352128468344</v>
+        <v>33.40352124728918</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5599382696461727</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0014301550552484</v>
+        <v>0.0014301551513873</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>45.10405205242138</v>
+        <v>45.10405202881413</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.22443952309385</v>
+        <v>16.22443944982156</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.4564191399267124</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>13.93816890486824</v>
+        <v>13.93816890775241</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>476.3940878282345</v>
+        <v>476.3940878282338</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>152</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>47.35160953445973</v>
+        <v>47.35160933602227</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.10430200231222</v>
+        <v>11.10430195638008</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.7802337605706574</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.400772741815649</v>
+        <v>1.400772740974454</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>60.78868716198352</v>
+        <v>60.78868714410726</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.20011139271191</v>
+        <v>16.20011141031293</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.3037742932108493</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.5184204952949485</v>
+        <v>0.5184204967370465</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>58.34177907658229</v>
+        <v>58.34177937626595</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.45368095559672</v>
+        <v>16.45368098300562</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.450181888168149</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>43.61479203807679</v>
+        <v>43.61479199911062</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>49.92852346018392</v>
+        <v>49.92852364383849</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.481116714517904</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1741045996310841</v>
+        <v>-0.1741045999435178</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>54.64787304063724</v>
+        <v>54.64787318540068</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>33.17188141048766</v>
+        <v>33.17188142979399</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.1947280560024797</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.6645011376424814</v>
+        <v>-0.6645011389644035</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>54.35215976944079</v>
+        <v>54.35215962498845</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>28.84073711932333</v>
+        <v>28.84073717960658</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.158514133372914</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.9639632257071638</v>
+        <v>-0.963963224385206</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>49.43217809854505</v>
+        <v>49.43217811180475</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>27.98759371865979</v>
+        <v>27.98759383390773</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.6452168589979339</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-1.588588773998094</v>
+        <v>-1.58858877423844</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>47.37334245576975</v>
+        <v>47.37334245143499</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.52282572285628</v>
+        <v>13.52282562233363</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.5882342702749326</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>25.20556947782829</v>
+        <v>25.20556947903</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>51.2411090555792</v>
+        <v>51.24110903408482</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.9346796623055</v>
+        <v>22.93467973216989</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3903580845066928</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>51.65400781449942</v>
+        <v>51.65400781223421</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>7.63316600810276</v>
+        <v>7.633166024504992</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>2.448835737686534</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>37.41460649908875</v>
+        <v>37.41460637498577</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>18.51483560138672</v>
+        <v>18.51483563103665</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.656443821053746</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>52.31951637530451</v>
+        <v>52.31951637459591</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>8.064490679535579</v>
+        <v>8.064490803115158</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>2.733612273361228</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>5.708419677203208</v>
+        <v>5.708419677323404</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>55.44962309923185</v>
+        <v>55.44962302674291</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>26.72143123462655</v>
+        <v>26.72143127604103</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5863235811745992</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.534243710774611</v>
+        <v>1.534243711495613</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>45.21522146617281</v>
+        <v>45.21522146812969</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>10.04215187339321</v>
+        <v>10.04215176125953</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.9664782276683432</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-12.17614973682719</v>
+        <v>-12.17614973370276</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>44.63241900006828</v>
+        <v>44.63241863391424</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>8.341395361994861</v>
+        <v>8.341395257583754</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6706850036822366</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.6900375520778192</v>
+        <v>0.6900375548418038</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>47.30882388330181</v>
+        <v>47.30882368929429</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>33.78076401580392</v>
+        <v>33.78076411955344</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5071619627032389</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.6562626399081606</v>
+        <v>0.6562626401965737</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>55.14734069551594</v>
+        <v>55.14734063633557</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>19.09916842795922</v>
+        <v>19.09916846383402</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.23910734439072</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>7.329285919117096</v>
+        <v>7.329285918395989</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>53.04926730859336</v>
+        <v>53.04926719054362</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>23.28141755937872</v>
+        <v>23.28141762529111</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.6774487725893804</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.08983058689745441</v>
+        <v>0.08983058698157539</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>387.5545965173487</v>
+        <v>387.5545965173492</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>32.4</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>56.89576343395816</v>
+        <v>56.8957633443066</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.29017033401312</v>
+        <v>16.29017039924022</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.182903369480411</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0582077357325422</v>
+        <v>0.0582077356724556</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>25.99341964798284</v>
+        <v>25.99341970638369</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>45.33118298914442</v>
+        <v>45.33118315185428</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3032416808382552</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>30.34719791964477</v>
+        <v>30.34719791552573</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>45.01532160705612</v>
+        <v>45.01532164553559</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>35.2488939890216</v>
+        <v>35.24889399323117</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.4375706557492224</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.7429178705640387</v>
+        <v>-0.7429178708043762</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>372.8513531235837</v>
+        <v>372.8513531235831</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>35.1</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>20.90043540557235</v>
+        <v>20.90043557156204</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>37.84849333884772</v>
+        <v>37.84849332960141</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6906092545194831</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.2067563951740039</v>
+        <v>-0.2067563957147791</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>38.48264195078113</v>
+        <v>38.48264171967865</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>24.03951375320212</v>
+        <v>24.0395138402084</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.5075217280688077</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.6425783365227451</v>
+        <v>0.6425783368832554</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>54.11986194121604</v>
+        <v>54.11986167121862</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>15.12464393489284</v>
+        <v>15.12464388776239</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.07401027846782129</v>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>336.51942115376</v>
+        <v>336.5194211537602</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>68</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>25.06710655206301</v>
+        <v>25.06710662489561</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>30.21164487737191</v>
+        <v>30.21164489097736</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>3.610773626878688</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0265962107606881</v>
+        <v>-0.026596210856822</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>330.4019181659302</v>
+        <v>330.4019181659324</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>0</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>23.10910075921979</v>
+        <v>23.1091009095545</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.03699505527415</v>
+        <v>12.03699504761276</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-5.882050763963326</v>
+        <v>-5.882050764083494</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>328.4508874188894</v>
+        <v>328.4508874188895</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>71.90000000000001</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>58.10563961013701</v>
+        <v>58.10563949033712</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.43545072926095</v>
+        <v>17.43545065805319</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.5736383681643722</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.8632352686326438</v>
+        <v>0.8632352688008764</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.86182570795097</v>
+        <v>47.86182573494251</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.26833841371437</v>
+        <v>17.26833840466432</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.5460593787290072</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-24.92779223118116</v>
+        <v>-24.92779223250308</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>326.3317708638371</v>
+        <v>326.331770863837</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>40.7</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>54.04339056152293</v>
+        <v>54.04339076782269</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.85901547461113</v>
+        <v>12.85901534908922</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.155151093987921</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0160754420700004</v>
+        <v>-0.0160754425987583</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>60.16187510250462</v>
+        <v>60.16187536131999</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>27.02695347443517</v>
+        <v>27.02695344652044</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.4668041039286125</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.5369390294277889</v>
+        <v>0.5369390283462305</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5113,7 +5113,7 @@
         <v>43.28448770294646</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.28426114487976</v>
+        <v>10.28426122988592</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.11149836238872</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.3231250056379406</v>
+        <v>0.323125005782144</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>311.9010234247981</v>
+        <v>311.901023424798</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>93</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>48.52396240007624</v>
+        <v>48.52396065766404</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>5.580613666799087</v>
+        <v>5.58061420205263</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.4393353859965352</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.8285801268576987</v>
+        <v>0.8285801733646814</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>47.15610161389711</v>
+        <v>47.15610159139001</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.3157228365921</v>
+        <v>19.31572296405096</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.071524287644398</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0886270891126706</v>
+        <v>0.0886270890165303</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>45.17589854604216</v>
+        <v>45.17589867804213</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.37786684539092</v>
+        <v>15.37786692718714</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.341645067125195</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.6155984224475235</v>
+        <v>0.6155984218466544</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>52.22053517459052</v>
+        <v>52.22053514886783</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>23.6186559827066</v>
+        <v>23.61865598222654</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.332262405207214</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.222928405739</v>
+        <v>49.22292853808494</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>17.71252835174026</v>
+        <v>17.71252839362713</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.227778012697675</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1468961361648818</v>
+        <v>0.1468961358043653</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>51.05934307415978</v>
+        <v>51.0593433107094</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>26.12438050794653</v>
+        <v>26.12438049301447</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.4846124356905155</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0266820713317251</v>
+        <v>0.0266820710553289</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>46.18124490769684</v>
+        <v>46.18124471149682</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>15.15317010055109</v>
+        <v>15.15317010220721</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7489362044903951</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>1.331329733949858</v>
+        <v>1.331329734670936</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>33.14581101112843</v>
+        <v>33.14581106507784</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>29.11968747946038</v>
+        <v>29.11968759366843</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.6038611477836315</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.4468606511579089</v>
+        <v>0.4468606546429177</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>27.66320177685313</v>
+        <v>27.6632016151332</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>37.63453746505432</v>
+        <v>37.63453747954928</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4480527717873906</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.6567083668883904</v>
+        <v>0.6567083673690934</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>271.0263759076125</v>
+        <v>271.0263759076129</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>25.5</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>49.6398151206168</v>
+        <v>49.63981554135609</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>31.34532795496529</v>
+        <v>31.34532806808877</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.2581483652302438</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.0561291824671429</v>
+        <v>-0.0561291825873173</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>267.0526903905856</v>
+        <v>267.0526903905848</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>37.95</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>30.35305298364742</v>
+        <v>30.35305290959268</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>12.14012057361857</v>
+        <v>12.14012058954953</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.071720830435555</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0958726522606874</v>
+        <v>-0.0958726522366545</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>255.4558240673253</v>
+        <v>255.4558240673252</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>92.90000000000001</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>50.33739465573956</v>
+        <v>50.33739461502287</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>13.73933934087768</v>
+        <v>13.73933924319254</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5751039035078224</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.2913641915979833</v>
+        <v>0.2913641921988509</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.24283705479002</v>
+        <v>52.24283621945295</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>14.49921384830902</v>
+        <v>14.49921387943165</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5548265515267909</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.1195131433275752</v>
+        <v>0.1195131434838089</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>41.53131316305589</v>
+        <v>41.53131298092942</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>16.1131398992769</v>
+        <v>16.11313989932438</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.3552683803288763</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.2115559010594885</v>
+        <v>0.2115559014920909</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>236.9843172392925</v>
+        <v>236.9843172392923</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>35.7</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>42.72470348661386</v>
+        <v>42.72470382863524</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>10.72970375519665</v>
+        <v>10.72970362184553</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.5972683625262174</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0903762533948541</v>
+        <v>0.09037625248153951</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.18868659681389</v>
+        <v>50.18868662677511</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.67989814541059</v>
+        <v>13.67989813241321</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.2002847541067448</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.312012911376657</v>
+        <v>-0.3120129119775203</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>226.7949030897586</v>
+        <v>226.7949030897587</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>36.85</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>44.39900535685848</v>
+        <v>44.39900539166531</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>35.821321189104</v>
+        <v>35.82132121452263</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.2747177275349578</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>52.11015844719259</v>
+        <v>52.11015844110335</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>8.893518663665803</v>
+        <v>8.893518684666871</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.7715106812434813</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>40.97751018254605</v>
+        <v>40.97751023002712</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>12.25905121525441</v>
+        <v>12.25905122467859</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.4265577258606749</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1961263014360004</v>
+        <v>-0.1961263016282817</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>43.27636943110653</v>
+        <v>43.27636890270136</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>10.97017256952574</v>
+        <v>10.9701731902514</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.6944112305375483</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0403910976742875</v>
+        <v>0.0403911022408763</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>205.4876869730767</v>
+        <v>205.4876869730768</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>73.59999999999999</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.84102864760256</v>
+        <v>46.84102871310257</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.5742295487741</v>
+        <v>14.57422958479083</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.1950710223370058</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.171986044302638</v>
+        <v>-0.171986044567024</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>200.0762819365945</v>
+        <v>200.0762819365937</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>33.55</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>51.5221376619051</v>
+        <v>51.52213764999456</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>7.360269190876881</v>
+        <v>7.360269027989748</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.6579849211788896</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.7715142106831939</v>
+        <v>0.7715142107192475</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>198.6874807893398</v>
+        <v>198.6874807893397</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>53.9</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>32.09203646378026</v>
+        <v>32.0920361131638</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>23.00490010909286</v>
+        <v>23.00490013329687</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.2552688175517914</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.08118454225323619</v>
+        <v>-0.0811845418927177</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.00215813912604</v>
+        <v>40.00215818443643</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>23.45723825138411</v>
+        <v>23.45723821509598</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.4122103442501256</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0666603632901908</v>
+        <v>-0.0666603633262431</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>42.96053927336681</v>
+        <v>42.96053908130381</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.17516194096955</v>
+        <v>16.17516192350935</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.4213970566760561</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>32.61790788655175</v>
+        <v>32.61790746514868</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>22.48847364367884</v>
+        <v>22.48847340730694</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4749274537933962</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.905784294454528</v>
+        <v>-0.9057842928922826</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>183.1426765614592</v>
+        <v>183.1426765614593</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>26.55</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>33.81625972607885</v>
+        <v>33.81625973098559</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.88077071031264</v>
+        <v>23.88077069871462</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.8699004936014489</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0051779720076648</v>
+        <v>0.0051779719956481</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>182.0902416818425</v>
+        <v>182.0902416818447</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>73.40000000000001</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>35.14603279959668</v>
+        <v>35.14603287232865</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>12.9991952328545</v>
+        <v>12.99919521481754</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.8592391715171215</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.2776834154936073</v>
+        <v>-0.2776834155176415</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>152.0196136673983</v>
+        <v>152.0196136673985</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>29.7</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>40.69329362252756</v>
+        <v>40.69329299083939</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>9.546972003825491</v>
+        <v>9.546972098378296</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.9326239046767693</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.008277347030397</v>
+        <v>0.0082773471505702</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>148.3111265158197</v>
+        <v>148.3111265158202</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>50.2</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>53.79102656575002</v>
+        <v>53.79102648848089</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>23.7295167014878</v>
+        <v>23.72951667486824</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.576402959485849</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0729292037159404</v>
+        <v>0.0729292037399748</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>143.3299578381896</v>
+        <v>143.3299578381904</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>166</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>39.38148185247181</v>
+        <v>39.38148167511107</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>17.34568048489323</v>
+        <v>17.34568047543972</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.8422734130354856</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0972389049233979</v>
+        <v>-0.0972389044427224</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>42.0098083505257</v>
+        <v>42.00980841928349</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>16.6172804228878</v>
+        <v>16.61728044359268</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.4252751215884963</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.9624517994744924</v>
+        <v>-0.962451800019593</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>132.9906000589774</v>
+        <v>132.9906000589775</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>45</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>41.88649615799974</v>
+        <v>41.88649566726436</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.57723380374128</v>
+        <v>12.5772338747424</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.4820937980073715</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0820299223075267</v>
+        <v>-0.0820299223315602</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>51.34344159048589</v>
+        <v>51.34344158604657</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.85018835316239</v>
+        <v>16.85018818063718</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.4189980584367054</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.871040951074016</v>
+        <v>-1.871040952035386</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>40.08590973427396</v>
+        <v>40.08590976189578</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>16.13356696693544</v>
+        <v>16.13356693298476</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.9289307309261348</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.1116062610792103</v>
+        <v>-0.1116062616800803</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>25.10859848809146</v>
+        <v>25.1085984252219</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>16.84372687654242</v>
+        <v>16.84372659628521</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.7619509147415975</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.2291016512376877</v>
+        <v>-0.2291016514299657</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>73.60965960820545</v>
+        <v>73.60965960820478</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>17.4</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>32.18038970384552</v>
+        <v>32.18038962323116</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>17.04639732297665</v>
+        <v>17.04639727265734</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>1.376083320559793</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.0434692336111838</v>
+        <v>-0.0434692335751275</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>